<commit_message>
refactor(content): migrate arena data to JSON and add translation skills
- Add Claude skills for translation pipelines (overview, implementation, tech-config)
- Migrate arena content from markdown to structured JSON format
- Add 10 new arena cases (nl2sql, credit-report, industrial-chain-graph, etc.)
- Replace nextjs.yml with deploy.yml workflow
- Add Python/shell scripts for docx-to-md and md-to-json conversion
- Consolidate page components by removing separate client files
- Export static arena data to public/data/ for optimized loading
- Remove obsolete video files and deprecated locale-redirect component

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19515" windowHeight="12255"/>
+    <workbookView windowWidth="31060" windowHeight="16060"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -244,7 +244,7 @@
         <rFont val="Arial"/>
         <charset val="134"/>
       </rPr>
-      <t>Claude Code + Kimi K2.5 + Metaso</t>
+      <t>Claude Code +Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5 + Metaso</t>
     </r>
   </si>
   <si>
@@ -405,7 +405,7 @@
         <rFont val="Arial"/>
         <charset val="134"/>
       </rPr>
-      <t>Lovable + Kimi K2.5 + Claude Code</t>
+      <t>Lovable + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5 + Claude Code</t>
     </r>
   </si>
   <si>
@@ -592,7 +592,7 @@
         <rFont val="Arial"/>
         <charset val="134"/>
       </rPr>
-      <t>LangChain + Kimi K2.5 + Pydantic + unstructured + Faiss</t>
+      <t>LangChain + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5  + Pydantic + unstructured + Faiss</t>
     </r>
   </si>
   <si>
@@ -708,7 +708,7 @@
         <rFont val="Arial"/>
         <charset val="134"/>
       </rPr>
-      <t>Claude Code + Kimi K2.5 + FFmpeg + FunASR + PaddleSpeech</t>
+      <t>Claude Code + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5  + FFmpeg + FunASR + PaddleSpeech</t>
     </r>
   </si>
   <si>
@@ -797,7 +797,7 @@
         <rFont val="Arial"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">BISHENG + Kimi K2.5 </t>
+      <t xml:space="preserve">BISHENG + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5 </t>
     </r>
   </si>
   <si>
@@ -1393,7 +1393,7 @@
         <rFont val="Arial"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">Coze + Kimi K2.5 </t>
+      <t xml:space="preserve">Coze + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5 </t>
     </r>
   </si>
   <si>
@@ -1440,18 +1440,7 @@
     </r>
   </si>
   <si>
-    <r>
-      <t>私部署版：</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">LangChain + Kimi K2.5 </t>
-    </r>
+    <t>私部署版：LangChain + Kimi K2.5/GLM-5/Minimax M2.5/Qwen 3.5  + Pydantic + unstructured + Faiss</t>
   </si>
   <si>
     <t>单条产业链图谱</t>
@@ -1555,6 +1544,12 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
@@ -1564,12 +1559,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10.5"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -2231,10 +2220,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2561,14 +2550,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="B2:M25"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
-    <col min="4" max="4" width="23.2583333333333" customWidth="1"/>
-    <col min="13" max="13" width="23.2583333333333" customWidth="1"/>
+    <col min="4" max="4" width="23.2596153846154" customWidth="1"/>
+    <col min="13" max="13" width="23.2596153846154" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" ht="15" customHeight="1"/>
-    <row r="3" ht="15" spans="2:13">
+    <row r="3" ht="34.75" spans="2:13">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -2606,7 +2595,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:13">
+    <row r="4" ht="17.55" spans="2:13">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -2616,83 +2605,83 @@
       <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M4" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="2:13">
+    <row r="5" ht="72" customHeight="1" spans="2:13">
       <c r="B5" s="3"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="6"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
     </row>
-    <row r="6" ht="114.75" spans="2:13">
+    <row r="6" ht="168.75" spans="2:13">
       <c r="B6">
         <v>2</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="L6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="7" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2706,28 +2695,28 @@
       <c r="D7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="6" t="s">
+      <c r="K7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L7" s="6" t="s">
+      <c r="L7" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M7" s="5" t="s">
@@ -2736,50 +2725,50 @@
     </row>
     <row r="8" spans="2:13">
       <c r="B8" s="3"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
     </row>
     <row r="9" ht="157.5" customHeight="1" spans="2:13">
       <c r="B9" s="3">
         <v>4</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>37</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M9" s="5" t="s">
@@ -2788,175 +2777,175 @@
     </row>
     <row r="10" spans="2:13">
       <c r="B10" s="3"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
     </row>
     <row r="11" ht="72" customHeight="1" spans="2:13">
       <c r="B11" s="3">
         <v>5</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>46</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="6" t="s">
+      <c r="J11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K11" s="6" t="s">
+      <c r="K11" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="6" t="s">
+      <c r="L11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M11" s="6" t="s">
+      <c r="M11" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" spans="2:13">
       <c r="B12" s="3"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
     </row>
     <row r="13" ht="129" customHeight="1" spans="2:13">
       <c r="B13" s="3">
         <v>6</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
         <v>49</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="H13" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L13" s="6" t="s">
+      <c r="L13" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:13">
+    <row r="14" ht="17.55" spans="2:13">
       <c r="B14" s="3"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
     </row>
     <row r="15" ht="114.75" customHeight="1" spans="2:13">
       <c r="B15" s="3">
         <v>7</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="6" t="s">
         <v>55</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G15" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="H15" s="6" t="s">
+      <c r="H15" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="6" t="s">
+      <c r="I15" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="J15" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K15" s="6" t="s">
+      <c r="K15" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L15" s="6" t="s">
+      <c r="L15" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M15" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="16" ht="14.25" spans="2:13">
+    <row r="16" ht="17.55" spans="2:13">
       <c r="B16" s="3"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="7"/>
     </row>
-    <row r="17" spans="2:13">
+    <row r="17" ht="17.55" spans="2:13">
       <c r="B17" s="3">
         <v>8</v>
       </c>
@@ -2966,269 +2955,269 @@
       <c r="D17" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="H17" s="6" t="s">
+      <c r="H17" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="I17" s="6" t="s">
+      <c r="I17" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L17" s="6" t="s">
+      <c r="L17" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M17" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="18" spans="2:13">
+    <row r="18" ht="17.55" spans="2:13">
       <c r="B18" s="3"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
     </row>
     <row r="19" ht="201" customHeight="1" spans="2:13">
       <c r="B19">
         <v>9</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="I19" s="6" t="s">
+      <c r="I19" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J19" s="6" t="s">
+      <c r="J19" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K19" s="6" t="s">
+      <c r="K19" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="L19" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M19" s="6" t="s">
+      <c r="M19" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="20" ht="72" spans="2:13">
+    <row r="20" ht="135.75" spans="2:13">
       <c r="B20">
         <v>10</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="H20" s="6" t="s">
+      <c r="H20" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I20" s="6" t="s">
+      <c r="I20" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J20" s="6" t="s">
+      <c r="J20" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="K20" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="M20" s="6" t="s">
+      <c r="M20" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="21" spans="2:13">
+    <row r="21" ht="17.55" spans="2:13">
       <c r="B21" s="3">
         <v>11</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>73</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I21" s="6" t="s">
+      <c r="I21" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J21" s="6" t="s">
+      <c r="J21" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="K21" s="6" t="s">
+      <c r="K21" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="7" t="s">
         <v>20</v>
       </c>
       <c r="M21" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="2:13">
+    <row r="22" ht="61" customHeight="1" spans="2:13">
       <c r="B22" s="3"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
-      <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
-      <c r="M22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="7"/>
+      <c r="M22" s="7"/>
     </row>
-    <row r="23" ht="157.5" spans="2:13">
+    <row r="23" ht="236.75" spans="2:13">
       <c r="B23">
         <v>12</v>
       </c>
-      <c r="C23" s="7" t="s">
+      <c r="C23" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J23" s="6" t="s">
+      <c r="J23" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K23" s="6" t="s">
+      <c r="K23" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L23" s="6" t="s">
+      <c r="L23" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M23" s="6" t="s">
+      <c r="M23" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="24" ht="86.25" spans="2:13">
+    <row r="24" ht="118.75" spans="2:13">
       <c r="B24">
         <v>13</v>
       </c>
-      <c r="C24" s="7" t="s">
+      <c r="C24" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="H24" s="6" t="s">
+      <c r="H24" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I24" s="6" t="s">
+      <c r="I24" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J24" s="6" t="s">
+      <c r="J24" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="K24" s="6" t="s">
+      <c r="K24" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="L24" s="6" t="s">
+      <c r="L24" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="M24" s="6" t="s">
+      <c r="M24" s="7" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="25" ht="29.25" spans="2:13">
+    <row r="25" ht="34.75" spans="2:13">
       <c r="B25">
         <v>14</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
-      <c r="H25" s="10"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
       <c r="I25" s="11"/>
       <c r="J25" s="11"/>
       <c r="K25" s="11"/>
       <c r="L25" s="11"/>
-      <c r="M25" s="10"/>
+      <c r="M25" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="96">
@@ -3354,7 +3343,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -3366,7 +3355,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>